<commit_message>
Fix aiService.isGreetingMessage export and ensure data persistence
</commit_message>
<xml_diff>
--- a/candidates_hiring.xlsx
+++ b/candidates_hiring.xlsx
@@ -397,27 +397,966 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:Q17"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
     <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="30.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="32.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
     <col min="12" max="12" width="22.83203125" customWidth="1"/>
     <col min="13" max="13" width="22.83203125" customWidth="1"/>
-    <col min="14" max="14" width="30.83203125" customWidth="1"/>
-    <col min="15" max="15" width="25.83203125" customWidth="1"/>
+    <col min="14" max="14" width="22.83203125" customWidth="1"/>
+    <col min="15" max="15" width="30.83203125" customWidth="1"/>
+    <col min="16" max="16" width="25.83203125" customWidth="1"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>S.No</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Candidate Name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>WhatsApp Phone</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Role Applied</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Work Mode</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Interview Mode</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Resume Received</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Portfolio / Drive / Social Link</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Candidate Status</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Interview Date &amp; Time</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Experience</v>
+      </c>
+      <c r="L1" t="str">
+        <v>City</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Resume Reminder Sent</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Interview 1hr Reminder</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Applied Date</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Last Message</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Candidate</v>
+      </c>
+      <c r="C2" t="str">
+        <v>+919876543211</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Influencer Collaboration</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Influencer Collaboration</v>
+      </c>
+      <c r="F2" t="str">
+        <v>In-Person (Indore Office)</v>
+      </c>
+      <c r="G2" t="str">
+        <v>PENDING</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Social: @tech_creator (45k)</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Applied</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Not Scheduled</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Preferred: Influencer Collaboration</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="M2" t="str">
+        <v>NO</v>
+      </c>
+      <c r="N2" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O2" t="str">
+        <v>14-Sept-2026, 2:30 pm</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Hello, I want to connect for Influencer Collaboration. My instagram is @tech_creator with 45k followers</v>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Candidate</v>
+      </c>
+      <c r="C3" t="str">
+        <v>+919876543210</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Video Editor</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Freelancer</v>
+      </c>
+      <c r="F3" t="str">
+        <v>In-Person (Indore Office)</v>
+      </c>
+      <c r="G3" t="str">
+        <v>PENDING</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v>Applied</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Not Scheduled</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Preferred: Freelancer</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="M3" t="str">
+        <v>NO</v>
+      </c>
+      <c r="N3" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O3" t="str">
+        <v>14-Sept-2026, 2:30 pm</v>
+      </c>
+      <c r="P3" t="str">
+        <v>Hi I am Rahul, I want to apply for video editor freelance work from home</v>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Arjun Meena</v>
+      </c>
+      <c r="C4" t="str">
+        <v>+918357977322</v>
+      </c>
+      <c r="D4" t="str">
+        <v>SEO &amp; AEO Expert</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Full-Time</v>
+      </c>
+      <c r="F4" t="str">
+        <v>In-Person (Indore Office)</v>
+      </c>
+      <c r="G4" t="str">
+        <v>YES</v>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v>Interview Scheduled</v>
+      </c>
+      <c r="J4" t="str">
+        <v>08-Sept-2026, 11:00 am</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Experienced (Full-Time)</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="M4" t="str">
+        <v>NO</v>
+      </c>
+      <c r="N4" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O4" t="str">
+        <v>07-Sept-2026, 1:26 pm</v>
+      </c>
+      <c r="P4" t="str">
+        <v>Great! See you at the interview. 👍 All the best! 😊</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>Auto-scheduled via WhatsApp AI: "Yes" (In-Person)</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Tanmay Jain</v>
+      </c>
+      <c r="C5" t="str">
+        <v>+919993297342</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Digital Marketing Manager</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Full-Time</v>
+      </c>
+      <c r="F5" t="str">
+        <v>In-Person (Indore Office)</v>
+      </c>
+      <c r="G5" t="str">
+        <v>YES</v>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v>Resume Received</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Not Scheduled</v>
+      </c>
+      <c r="K5" t="str">
+        <v>6 years</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="M5" t="str">
+        <v>NO</v>
+      </c>
+      <c r="N5" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O5" t="str">
+        <v>07-Sept-2026, 11:48 am</v>
+      </c>
+      <c r="P5" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hello Tanmay Jain! 😊
+Great news! Your profile and portfolio have been shortlisted by our HR team. 👏✨
+👉 Are you available to visit our Indore office (*103 Orange Business Park, Bhawarkua*) for an in-person practical interview tomorrow morning between *10:00 AM and 12:00 PM*? 🏢
+Please confirm (Yes / No or share your preferred time). 👍</v>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Shyama's house of snacks</v>
+      </c>
+      <c r="C6" t="str">
+        <v>+917693884339</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Digital Marketing Manager</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Full-Time</v>
+      </c>
+      <c r="F6" t="str">
+        <v>In-Person (Indore Office)</v>
+      </c>
+      <c r="G6" t="str">
+        <v>YES</v>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v>Interview Scheduled</v>
+      </c>
+      <c r="J6" t="str">
+        <v>05-Sept-2026, 11:00 am</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Fresher (Paid Internship)</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="M6" t="str">
+        <v>NO</v>
+      </c>
+      <c r="N6" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O6" t="str">
+        <v>04-Sept-2026, 2:28 pm</v>
+      </c>
+      <c r="P6" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dear Shyama's house of snacks! 🔄
+Your interview for the *Digital Marketing Manager* position at *BrandSetu Digital* has been *rescheduled successfully*.
+📅 *Updated Date &amp; Time:* Sat, 5 Sept, 2026, 11:00 am
+📍 *Office Address:* 103 Orange Business Park, Bhawarkua Main Road, Near Apple Hospital, Transport Nagar, Indore (M.P.) - 452014
+📌 Please bring your updated Resume and work samples/portfolio.
+For any questions or directions, reply here or contact us at +91 9329232025.
+See you then! 👍
+- HR Team, BrandSetu Digital</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>Auto-scheduled via WhatsApp AI: "ok sir" (In-Person)</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>BrandSetuDigital</v>
+      </c>
+      <c r="C7" t="str">
+        <v>+919669765911</v>
+      </c>
+      <c r="D7" t="str">
+        <v>General Applicant</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Full-Time</v>
+      </c>
+      <c r="F7" t="str">
+        <v>In-Person (Indore Office)</v>
+      </c>
+      <c r="G7" t="str">
+        <v>PENDING</v>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v>Resume Pending</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Not Scheduled</v>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="M7" t="str">
+        <v>YES</v>
+      </c>
+      <c r="N7" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O7" t="str">
+        <v>04-Sept-2026, 2:33 pm</v>
+      </c>
+      <c r="P7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Namaste BrandSetuDigital! 👋
+BrandSetu Digital me *General Applicant* position ke liye aapke interest ke liye dhanyawad. Humein abhi tak aapka updated *Resume / Portfolio* receive nahi hua hai. 📄
+👉 Kripya apna Resume (PDF) ya Portfolio link yahan share karein taaki hum aapka interview schedule kar sakein. 🚀
+- HR Team, BrandSetu Digital (+91 9329232025)</v>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Mohit 🎬</v>
+      </c>
+      <c r="C8" t="str">
+        <v>+917470584339</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Video Editor</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Full-Time</v>
+      </c>
+      <c r="F8" t="str">
+        <v>In-Person (Indore Office)</v>
+      </c>
+      <c r="G8" t="str">
+        <v>YES</v>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v>Resume Received</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Not Scheduled</v>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="M8" t="str">
+        <v>NO</v>
+      </c>
+      <c r="N8" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O8" t="str">
+        <v>20-Aug-2026, 4:31 pm</v>
+      </c>
+      <c r="P8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hello Mohit! 😊
+Aapki profile aur portfolio HR team dwara shortlist kar li gayi hai. 👏✨
+👉 Kya aap kal morning me *10:00 AM se 12:00 PM* ke beech hamare Indore office (*103 Orange Business Park, Bhawarkua*) in-person interview ke liye aa sakte hain? 🏢
+Kripya confirm karein (Haan / Nahi ya apna suitable time batayein). 👍</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>Auto-scheduled via WhatsApp AI: "Tomorrow morning 12 pm"</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>manshi</v>
+      </c>
+      <c r="C9" t="str">
+        <v>+917828966773</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Digital Marketing Manager</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Full-Time</v>
+      </c>
+      <c r="F9" t="str">
+        <v>In-Person (Indore Office)</v>
+      </c>
+      <c r="G9" t="str">
+        <v>PENDING</v>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v>Resume Pending</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Not Scheduled</v>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="M9" t="str">
+        <v>YES</v>
+      </c>
+      <c r="N9" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O9" t="str">
+        <v>04-Sept-2026, 2:27 pm</v>
+      </c>
+      <c r="P9" t="str" xml:space="preserve">
+        <v xml:space="preserve">Namaste manshi! 👋
+BrandSetu Digital me *Digital Marketing Manager* position ke liye aapke interest ke liye dhanyawad. Humein abhi tak aapka updated *Resume / Portfolio* receive nahi hua hai. 📄
+👉 Kripya apna Resume (PDF) ya Portfolio link yahan share karein taaki hum aapka interview schedule kar sakein. 🚀
+- HR Team, BrandSetu Digital (+91 9329232025)</v>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Aabid</v>
+      </c>
+      <c r="C10" t="str">
+        <v>+917869724727</v>
+      </c>
+      <c r="D10" t="str">
+        <v>AI Video Expert</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Full-Time</v>
+      </c>
+      <c r="F10" t="str">
+        <v>In-Person (Indore Office)</v>
+      </c>
+      <c r="G10" t="str">
+        <v>YES</v>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v>Interview Scheduled</v>
+      </c>
+      <c r="J10" t="str">
+        <v>04-Sept-2026, 2:00 pm</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Experienced (Full-Time)</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="M10" t="str">
+        <v>NO</v>
+      </c>
+      <c r="N10" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O10" t="str">
+        <v>04-Sept-2026, 2:15 pm</v>
+      </c>
+      <c r="P10" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dear Aabid! 🎉
+Your interview for the *AI Video Expert* position at *BrandSetu Digital* has been scheduled successfully.
+📅 *Date &amp; Time:* Fri, 4 Sept, 2026, 02:00 pm
+📍 *Office Address:* 103 Orange Business Park, Bhawarkua Main Road, Near Apple Hospital, Transport Nagar, Indore (M.P.) - 452014
+📌 Please bring your updated Resume and work samples/portfolio.
+For any questions or directions, reply here or contact us at +91 9329232025.
+Best of luck! 👍
+- HR Team, BrandSetu Digital</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>Auto-scheduled via WhatsApp AI: "Today 2 PM" (In-Person)</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Nancy Ajmera</v>
+      </c>
+      <c r="C11" t="str">
+        <v>+38899686625461</v>
+      </c>
+      <c r="D11" t="str">
+        <v>General Applicant</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Full-Time</v>
+      </c>
+      <c r="F11" t="str">
+        <v>In-Person (Indore Office)</v>
+      </c>
+      <c r="G11" t="str">
+        <v>PENDING</v>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v>Applied</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Not Scheduled</v>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="M11" t="str">
+        <v>YES</v>
+      </c>
+      <c r="N11" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O11" t="str">
+        <v>03-Sept-2026, 5:03 pm</v>
+      </c>
+      <c r="P11" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hello Nancy! 😊
+Welcome to Brand Setu Digital! 🎉
+We are actively hiring for:
+1️⃣ 🎬 *Video Editor*
+2️⃣ 🤖 *AI Video Expert*
+3️⃣ 🎨 *Graphic Designer*
+4️⃣ 🔎 *SEO &amp; AEO Expert*
+5️⃣ 📱 *Social Media Manager*
+6️⃣ 📢 *Digital Marketing Manager*
+👉 Which **position/role** would you like to apply for? (Please reply with number 1 to 6 or the role name) 📝</v>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Unnat</v>
+      </c>
+      <c r="C12" t="str">
+        <v>+278880866857060</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Video Editor</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Full-Time</v>
+      </c>
+      <c r="F12" t="str">
+        <v>In-Person (Indore Office)</v>
+      </c>
+      <c r="G12" t="str">
+        <v>YES</v>
+      </c>
+      <c r="H12" t="str">
+        <v>https://corrra.com/@unnatportfolio</v>
+      </c>
+      <c r="I12" t="str">
+        <v>Interview Scheduled</v>
+      </c>
+      <c r="J12" t="str">
+        <v>04-Sept-2026, 4:00 pm</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Experienced (Full-Time)</v>
+      </c>
+      <c r="L12" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="M12" t="str">
+        <v>NO</v>
+      </c>
+      <c r="N12" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O12" t="str">
+        <v>03-Sept-2026, 3:58 pm</v>
+      </c>
+      <c r="P12" t="str">
+        <v>4 sep friday</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>Auto-scheduled via WhatsApp AI: "4 sep friday"</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Arjun Meena</v>
+      </c>
+      <c r="C13" t="str">
+        <v>+919329232025</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Video Editor</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Full-Time</v>
+      </c>
+      <c r="F13" t="str">
+        <v>In-Person (Indore Office)</v>
+      </c>
+      <c r="G13" t="str">
+        <v>YES</v>
+      </c>
+      <c r="H13" t="str">
+        <v>https://drive.google.com/drive/folders/sample_portfolio</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Interview Scheduled</v>
+      </c>
+      <c r="J13" t="str">
+        <v>04-Sept-2026, 2:00 pm</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Fresher (Paid Internship)</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="M13" t="str">
+        <v>NO</v>
+      </c>
+      <c r="N13" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O13" t="str">
+        <v>03-Sept-2026, 3:35 pm</v>
+      </c>
+      <c r="P13" t="str">
+        <v>Kal dopahar 2 baje</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>Test auto schedule</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Arjun Meena</v>
+      </c>
+      <c r="C14" t="str">
+        <v>+114405211672638</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Video Editor</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Full-Time</v>
+      </c>
+      <c r="F14" t="str">
+        <v>In-Person (Indore Office)</v>
+      </c>
+      <c r="G14" t="str">
+        <v>YES</v>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v>Interview Scheduled</v>
+      </c>
+      <c r="J14" t="str">
+        <v>03-Sept-2026, 5:00 pm</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Fresher (Paid Internship)</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="M14" t="str">
+        <v>NO</v>
+      </c>
+      <c r="N14" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O14" t="str">
+        <v>03-Sept-2026, 2:29 pm</v>
+      </c>
+      <c r="P14" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hello Arjun! 😊
+Your interview is already confirmed for *Thu, 3 Sept, 05:00 pm* at 103 Orange Business Park, Bhawarkua, Indore. We look forward to meeting you! 😊📍</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>Auto-scheduled via WhatsApp AI: "Today 5:3 mint pe mera interview resedule kr do"</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>manisha</v>
+      </c>
+      <c r="C15" t="str">
+        <v>+917879010084</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Video Editor</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Full-Time</v>
+      </c>
+      <c r="F15" t="str">
+        <v>In-Person (Indore Office)</v>
+      </c>
+      <c r="G15" t="str">
+        <v>PENDING</v>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v>Resume Pending</v>
+      </c>
+      <c r="J15" t="str">
+        <v>Not Scheduled</v>
+      </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="M15" t="str">
+        <v>YES</v>
+      </c>
+      <c r="N15" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O15" t="str">
+        <v>20-Aug-2026, 3:49 pm</v>
+      </c>
+      <c r="P15" t="str">
+        <v>Hello manisha! 😊 Please share your updated *Resume (PDF)* or Portfolio/Drive link here so we can proceed with your application! 📄💼</v>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Annushka</v>
+      </c>
+      <c r="C16" t="str">
+        <v>+919039193109</v>
+      </c>
+      <c r="D16" t="str">
+        <v>General Applicant</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Full-Time</v>
+      </c>
+      <c r="F16" t="str">
+        <v>In-Person (Indore Office)</v>
+      </c>
+      <c r="G16" t="str">
+        <v>PENDING</v>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v>Resume Pending</v>
+      </c>
+      <c r="J16" t="str">
+        <v>Not Scheduled</v>
+      </c>
+      <c r="K16" t="str">
+        <v/>
+      </c>
+      <c r="L16" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="M16" t="str">
+        <v>YES</v>
+      </c>
+      <c r="N16" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O16" t="str">
+        <v>10-Sept-2026, 12:45 pm</v>
+      </c>
+      <c r="P16" t="str">
+        <v>Hiiii</v>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>सौमित्र</v>
+      </c>
+      <c r="C17" t="str">
+        <v>+919770477701</v>
+      </c>
+      <c r="D17" t="str">
+        <v>AI Video Expert</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Full-Time</v>
+      </c>
+      <c r="F17" t="str">
+        <v>In-Person (Indore Office)</v>
+      </c>
+      <c r="G17" t="str">
+        <v>PENDING</v>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v>Not Interested</v>
+      </c>
+      <c r="J17" t="str">
+        <v>Not Scheduled</v>
+      </c>
+      <c r="K17" t="str">
+        <v/>
+      </c>
+      <c r="L17" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="M17" t="str">
+        <v>YES</v>
+      </c>
+      <c r="N17" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O17" t="str">
+        <v>12-Sept-2026, 2:49 pm</v>
+      </c>
+      <c r="P17" t="str">
+        <v>Hi</v>
+      </c>
+      <c r="Q17" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: smart excel phone extraction and meta webhook status tracking
</commit_message>
<xml_diff>
--- a/candidates_hiring.xlsx
+++ b/candidates_hiring.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q52"/>
+  <dimension ref="A1:Q53"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -470,7 +470,7 @@
         <v>Notes</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2">
         <v>1</v>
       </c>
@@ -516,8 +516,11 @@
       <c r="O2" t="str">
         <v>16-Sept-2026, 12:04 pm</v>
       </c>
-      <c r="P2" t="str">
-        <v>https://garimanamdevportfolio.my.canva.site/creative-portfolio GarimaNamdevResume.pdf</v>
+      <c r="P2" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hello Garima Namdev! 😊
+Great news! Your profile and portfolio have been shortlisted by our HR team. 👏✨
+👉 Are you available to visit our Indore office (*103 Orange Business Park, Bhawarkua*) for an in-person practical interview tomorrow morning between *10:00 AM and 12:00 PM*? 🏢
+Please confirm (Yes / No or share your preferred time). 👍</v>
       </c>
       <c r="Q2" t="str">
         <v/>
@@ -3315,9 +3318,84 @@
         <v/>
       </c>
     </row>
+    <row r="53" xml:space="preserve">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Candidate</v>
+      </c>
+      <c r="C53" t="str">
+        <v>+918085513390</v>
+      </c>
+      <c r="D53" t="str">
+        <v>General Applicant</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Full-Time</v>
+      </c>
+      <c r="F53" t="str">
+        <v>In-Person (Indore Office)</v>
+      </c>
+      <c r="G53" t="str">
+        <v>PENDING</v>
+      </c>
+      <c r="H53" t="str">
+        <v/>
+      </c>
+      <c r="I53" t="str">
+        <v>Campaign Sent</v>
+      </c>
+      <c r="J53" t="str">
+        <v>Not Scheduled</v>
+      </c>
+      <c r="K53" t="str">
+        <v/>
+      </c>
+      <c r="L53" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="M53" t="str">
+        <v>NO</v>
+      </c>
+      <c r="N53" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O53" t="str">
+        <v>16-Sept-2026, 12:17 pm</v>
+      </c>
+      <c r="P53" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hello! 👋_x000d_
+_x000d_
+Brand Setu Digital is expanding its Creative &amp; Marketing Team! 🚀_x000d_
+_x000d_
+We are currently hiring for multiple positions:_x000d_
+_x000d_
+1️⃣ Video Editor – Reels / YouTube 🎬_x000d_
+2️⃣ AI Video Expert – AI Tools / Prompting 🤖_x000d_
+3️⃣ Graphic Designer – Photoshop / Figma 🎨_x000d_
+4️⃣ SEO &amp; AEO Expert 🔎_x000d_
+5️⃣ Social Media Manager 📱_x000d_
+6️⃣ Digital Marketing Manager 📢_x000d_
+7️⃣ Influencer Collaboration ✨_x000d_
+_x000d_
+💼 Full-Time | Work From Home | Freelance opportunities are available._x000d_
+_x000d_
+If you’re interested, please share your updated Resume (PDF) and mention which position you are applying for._x000d_
+_x000d_
+👉 Example: “I’m applying for Position 1 – Video Editor.”_x000d_
+_x000d_
+If you’re interested in multiple positions, you can mention all the positions you’d like to apply for._x000d_
+_x000d_
+Our HR team will review your profile and get back to you with the next steps. 😊</v>
+      </c>
+      <c r="Q53" t="str">
+        <v>Outreach campaign broadcast sent</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q52"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q53"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(mongo): prevent immutable _id update in background sync
</commit_message>
<xml_diff>
--- a/candidates_hiring.xlsx
+++ b/candidates_hiring.xlsx
@@ -579,7 +579,7 @@
         <v/>
       </c>
     </row>
-    <row r="4">
+    <row r="4" xml:space="preserve">
       <c r="A4">
         <v>3</v>
       </c>
@@ -625,8 +625,11 @@
       <c r="O4" t="str">
         <v>16-Sept-2026, 11:54 am</v>
       </c>
-      <c r="P4" t="str">
-        <v>https://garimanamdevportfolio.my.canva.site/creative-portfolio GarimaNamdevResume.pdf</v>
+      <c r="P4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hello Garima Namdev! 😊
+Great news! Your profile and portfolio have been shortlisted by our HR team. 👏✨
+👉 Are you available to visit our Indore office (*103 Orange Business Park, Bhawarkua*) for an in-person practical interview tomorrow morning between *10:00 AM and 12:00 PM*? 🏢
+Please confirm (Yes / No or share your preferred time). 👍</v>
       </c>
       <c r="Q4" t="str">
         <v/>
@@ -3173,7 +3176,7 @@
         <v/>
       </c>
       <c r="I50" t="str">
-        <v>Applied</v>
+        <v>Resume Pending</v>
       </c>
       <c r="J50" t="str">
         <v>Not Scheduled</v>
@@ -3185,7 +3188,7 @@
         <v>Indore</v>
       </c>
       <c r="M50" t="str">
-        <v>NO</v>
+        <v>YES</v>
       </c>
       <c r="N50" t="str">
         <v>NO</v>
@@ -3194,8 +3197,10 @@
         <v>16-Sept-2026, 9:34 am</v>
       </c>
       <c r="P50" t="str" xml:space="preserve">
-        <v xml:space="preserve">Thank you for sharing your CV! 📄✨ 
-Our team is reviewing your profile and work samples. We will connect with you shortly for the next steps! 👍</v>
+        <v xml:space="preserve">Dear Anjali! 👋
+Thank you for your interest in joining *BrandSetu Digital* for the *Influencer Collaboration* position. We noticed we haven't received your updated *Resume / Portfolio* yet. 📄
+👉 Please share your Resume (PDF) or Portfolio link here so we can proceed with scheduling your interview. 🚀
+- HR Team, BrandSetu Digital (+91 9329232025 / +91 9669765911)</v>
       </c>
       <c r="Q50" t="str">
         <v/>

</xml_diff>